<commit_message>
BLP, BPP, BSFVBP extend past 2050
</commit_message>
<xml_diff>
--- a/InputData/trans/BLP/BAU LCFS Perc.xlsx
+++ b/InputData/trans/BLP/BAU LCFS Perc.xlsx
@@ -1,31 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganM\Documents\eps-us\InputData\trans\BLP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\eps-mexico\InputData\trans\BLP\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8CD1D8E-6AA8-44E0-AA86-C658CC0E2C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="BLP" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -68,10 +59,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.0000"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -638,49 +626,45 @@
       <alignment wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="63">
     <cellStyle name="20% - Accent1" xfId="25" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent1 2" xfId="50"/>
+    <cellStyle name="20% - Accent1 2" xfId="50" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="20% - Accent2" xfId="28" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2 2" xfId="52"/>
+    <cellStyle name="20% - Accent2 2" xfId="52" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="20% - Accent3" xfId="31" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3 2" xfId="54"/>
+    <cellStyle name="20% - Accent3 2" xfId="54" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
     <cellStyle name="20% - Accent4" xfId="34" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4 2" xfId="56"/>
+    <cellStyle name="20% - Accent4 2" xfId="56" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
     <cellStyle name="20% - Accent5" xfId="37" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5 2" xfId="58"/>
+    <cellStyle name="20% - Accent5 2" xfId="58" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
     <cellStyle name="20% - Accent6" xfId="40" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6 2" xfId="60"/>
+    <cellStyle name="20% - Accent6 2" xfId="60" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
     <cellStyle name="40% - Accent1" xfId="26" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1 2" xfId="51"/>
+    <cellStyle name="40% - Accent1 2" xfId="51" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
     <cellStyle name="40% - Accent2" xfId="29" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2 2" xfId="53"/>
+    <cellStyle name="40% - Accent2 2" xfId="53" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
     <cellStyle name="40% - Accent3" xfId="32" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3 2" xfId="55"/>
+    <cellStyle name="40% - Accent3 2" xfId="55" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
     <cellStyle name="40% - Accent4" xfId="35" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4 2" xfId="57"/>
+    <cellStyle name="40% - Accent4 2" xfId="57" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
     <cellStyle name="40% - Accent5" xfId="38" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5 2" xfId="59"/>
+    <cellStyle name="40% - Accent5 2" xfId="59" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
     <cellStyle name="40% - Accent6" xfId="41" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6 2" xfId="61"/>
-    <cellStyle name="60% - Accent1 2" xfId="43"/>
-    <cellStyle name="60% - Accent2 2" xfId="44"/>
-    <cellStyle name="60% - Accent3 2" xfId="45"/>
-    <cellStyle name="60% - Accent4 2" xfId="46"/>
-    <cellStyle name="60% - Accent5 2" xfId="47"/>
-    <cellStyle name="60% - Accent6 2" xfId="48"/>
+    <cellStyle name="40% - Accent6 2" xfId="61" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
+    <cellStyle name="60% - Accent1 2" xfId="43" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
+    <cellStyle name="60% - Accent2 2" xfId="44" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
+    <cellStyle name="60% - Accent3 2" xfId="45" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
+    <cellStyle name="60% - Accent4 2" xfId="46" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
+    <cellStyle name="60% - Accent5 2" xfId="47" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
+    <cellStyle name="60% - Accent6 2" xfId="48" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
     <cellStyle name="Accent1" xfId="24" builtinId="29" customBuiltin="1"/>
     <cellStyle name="Accent2" xfId="27" builtinId="33" customBuiltin="1"/>
     <cellStyle name="Accent3" xfId="30" builtinId="37" customBuiltin="1"/>
@@ -688,29 +672,29 @@
     <cellStyle name="Accent5" xfId="36" builtinId="45" customBuiltin="1"/>
     <cellStyle name="Accent6" xfId="39" builtinId="49" customBuiltin="1"/>
     <cellStyle name="Bad" xfId="14" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Body: normal cell" xfId="4"/>
-    <cellStyle name="Body: normal cell 2" xfId="62"/>
+    <cellStyle name="Body: normal cell" xfId="4" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
+    <cellStyle name="Body: normal cell 2" xfId="62" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
     <cellStyle name="Calculation" xfId="17" builtinId="22" customBuiltin="1"/>
     <cellStyle name="Check Cell" xfId="19" builtinId="23" customBuiltin="1"/>
     <cellStyle name="Explanatory Text" xfId="22" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Font: Calibri, 9pt regular" xfId="6"/>
-    <cellStyle name="Footnotes: top row" xfId="2"/>
+    <cellStyle name="Font: Calibri, 9pt regular" xfId="6" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
+    <cellStyle name="Footnotes: top row" xfId="2" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
     <cellStyle name="Good" xfId="13" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Header: bottom row" xfId="5"/>
+    <cellStyle name="Header: bottom row" xfId="5" xr:uid="{00000000-0005-0000-0000-00002D000000}"/>
     <cellStyle name="Heading 1" xfId="9" builtinId="16" customBuiltin="1"/>
     <cellStyle name="Heading 2" xfId="10" builtinId="17" customBuiltin="1"/>
     <cellStyle name="Heading 3" xfId="11" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Heading 4" xfId="12" builtinId="19" customBuiltin="1"/>
     <cellStyle name="Input" xfId="15" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="18" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral 2" xfId="42"/>
+    <cellStyle name="Neutral 2" xfId="42" xr:uid="{00000000-0005-0000-0000-000034000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
     <cellStyle name="Note" xfId="21" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Note 2" xfId="49"/>
+    <cellStyle name="Note 2" xfId="49" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
     <cellStyle name="Output" xfId="16" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Parent row" xfId="3"/>
-    <cellStyle name="Table title" xfId="7"/>
+    <cellStyle name="Parent row" xfId="3" xr:uid="{00000000-0005-0000-0000-00003A000000}"/>
+    <cellStyle name="Table title" xfId="7" xr:uid="{00000000-0005-0000-0000-00003B000000}"/>
     <cellStyle name="Title" xfId="8" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="23" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="20" builtinId="11" customBuiltin="1"/>
@@ -729,9 +713,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -769,9 +753,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -806,7 +790,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -841,7 +825,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1014,60 +998,57 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="2" max="2" width="56.73046875" customWidth="1"/>
+    <col min="2" max="2" width="56.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="B4" s="5"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1079,212 +1060,330 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AJ2"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:BB2"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="1" max="1" width="15.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:54" x14ac:dyDescent="0.75">
       <c r="B1">
         <v>2020</v>
       </c>
-      <c r="C1" s="4">
+      <c r="C1">
         <v>2021</v>
       </c>
-      <c r="D1" s="4">
+      <c r="D1">
         <v>2022</v>
       </c>
-      <c r="E1" s="4">
+      <c r="E1">
         <v>2023</v>
       </c>
-      <c r="F1" s="4">
+      <c r="F1">
         <v>2024</v>
       </c>
-      <c r="G1" s="4">
+      <c r="G1">
         <v>2025</v>
       </c>
-      <c r="H1" s="4">
+      <c r="H1">
         <v>2026</v>
       </c>
-      <c r="I1" s="4">
+      <c r="I1">
         <v>2027</v>
       </c>
-      <c r="J1" s="4">
+      <c r="J1">
         <v>2028</v>
       </c>
-      <c r="K1" s="4">
+      <c r="K1">
         <v>2029</v>
       </c>
-      <c r="L1" s="4">
+      <c r="L1">
         <v>2030</v>
       </c>
-      <c r="M1" s="4">
+      <c r="M1">
         <v>2031</v>
       </c>
-      <c r="N1" s="4">
+      <c r="N1">
         <v>2032</v>
       </c>
-      <c r="O1" s="4">
+      <c r="O1">
         <v>2033</v>
       </c>
-      <c r="P1" s="4">
+      <c r="P1">
         <v>2034</v>
       </c>
-      <c r="Q1" s="4">
+      <c r="Q1">
         <v>2035</v>
       </c>
-      <c r="R1" s="4">
+      <c r="R1">
         <v>2036</v>
       </c>
-      <c r="S1" s="4">
+      <c r="S1">
         <v>2037</v>
       </c>
-      <c r="T1" s="4">
+      <c r="T1">
         <v>2038</v>
       </c>
-      <c r="U1" s="4">
+      <c r="U1">
         <v>2039</v>
       </c>
-      <c r="V1" s="4">
+      <c r="V1">
         <v>2040</v>
       </c>
-      <c r="W1" s="4">
+      <c r="W1">
         <v>2041</v>
       </c>
-      <c r="X1" s="4">
+      <c r="X1">
         <v>2042</v>
       </c>
-      <c r="Y1" s="4">
+      <c r="Y1">
         <v>2043</v>
       </c>
-      <c r="Z1" s="4">
+      <c r="Z1">
         <v>2044</v>
       </c>
-      <c r="AA1" s="4">
+      <c r="AA1">
         <v>2045</v>
       </c>
-      <c r="AB1" s="4">
+      <c r="AB1">
         <v>2046</v>
       </c>
-      <c r="AC1" s="4">
+      <c r="AC1">
         <v>2047</v>
       </c>
-      <c r="AD1" s="4">
+      <c r="AD1">
         <v>2048</v>
       </c>
-      <c r="AE1" s="4">
+      <c r="AE1">
         <v>2049</v>
       </c>
-      <c r="AF1" s="4">
+      <c r="AF1">
         <v>2050</v>
       </c>
+      <c r="AG1">
+        <v>2051</v>
+      </c>
+      <c r="AH1">
+        <v>2052</v>
+      </c>
+      <c r="AI1">
+        <v>2053</v>
+      </c>
+      <c r="AJ1">
+        <v>2054</v>
+      </c>
+      <c r="AK1">
+        <v>2055</v>
+      </c>
+      <c r="AL1">
+        <v>2056</v>
+      </c>
+      <c r="AM1">
+        <v>2057</v>
+      </c>
+      <c r="AN1">
+        <v>2058</v>
+      </c>
+      <c r="AO1">
+        <v>2059</v>
+      </c>
+      <c r="AP1">
+        <v>2060</v>
+      </c>
+      <c r="AQ1">
+        <v>2061</v>
+      </c>
+      <c r="AR1">
+        <v>2062</v>
+      </c>
+      <c r="AS1">
+        <v>2063</v>
+      </c>
+      <c r="AT1">
+        <v>2064</v>
+      </c>
+      <c r="AU1">
+        <v>2065</v>
+      </c>
+      <c r="AV1">
+        <v>2066</v>
+      </c>
+      <c r="AW1">
+        <v>2067</v>
+      </c>
+      <c r="AX1">
+        <v>2068</v>
+      </c>
+      <c r="AY1">
+        <v>2069</v>
+      </c>
+      <c r="AZ1">
+        <v>2070</v>
+      </c>
     </row>
-    <row r="2" spans="1:36" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:54" ht="29.5" x14ac:dyDescent="0.75">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="7">
-        <v>0</v>
-      </c>
-      <c r="C2" s="7">
-        <v>0</v>
-      </c>
-      <c r="D2" s="7">
-        <v>0</v>
-      </c>
-      <c r="E2" s="7">
-        <v>0</v>
-      </c>
-      <c r="F2" s="7">
-        <v>0</v>
-      </c>
-      <c r="G2" s="7">
-        <v>0</v>
-      </c>
-      <c r="H2" s="7">
-        <v>0</v>
-      </c>
-      <c r="I2" s="7">
-        <v>0</v>
-      </c>
-      <c r="J2" s="7">
-        <v>0</v>
-      </c>
-      <c r="K2" s="7">
-        <v>0</v>
-      </c>
-      <c r="L2" s="7">
-        <v>0</v>
-      </c>
-      <c r="M2" s="7">
-        <v>0</v>
-      </c>
-      <c r="N2" s="7">
-        <v>0</v>
-      </c>
-      <c r="O2" s="7">
-        <v>0</v>
-      </c>
-      <c r="P2" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="7">
-        <v>0</v>
-      </c>
-      <c r="R2" s="7">
-        <v>0</v>
-      </c>
-      <c r="S2" s="7">
-        <v>0</v>
-      </c>
-      <c r="T2" s="7">
-        <v>0</v>
-      </c>
-      <c r="U2" s="7">
-        <v>0</v>
-      </c>
-      <c r="V2" s="7">
-        <v>0</v>
-      </c>
-      <c r="W2" s="7">
-        <v>0</v>
-      </c>
-      <c r="X2" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AG2" s="3"/>
-      <c r="AH2" s="3"/>
-      <c r="AI2" s="3"/>
-      <c r="AJ2" s="3"/>
+      <c r="B2" s="3">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3">
+        <v>0</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3">
+        <v>0</v>
+      </c>
+      <c r="F2" s="3">
+        <v>0</v>
+      </c>
+      <c r="G2" s="3">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3">
+        <v>0</v>
+      </c>
+      <c r="J2" s="3">
+        <v>0</v>
+      </c>
+      <c r="K2" s="3">
+        <v>0</v>
+      </c>
+      <c r="L2" s="3">
+        <v>0</v>
+      </c>
+      <c r="M2" s="3">
+        <v>0</v>
+      </c>
+      <c r="N2" s="3">
+        <v>0</v>
+      </c>
+      <c r="O2" s="3">
+        <v>0</v>
+      </c>
+      <c r="P2" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="3">
+        <v>0</v>
+      </c>
+      <c r="R2" s="3">
+        <v>0</v>
+      </c>
+      <c r="S2" s="3">
+        <v>0</v>
+      </c>
+      <c r="T2" s="3">
+        <v>0</v>
+      </c>
+      <c r="U2" s="3">
+        <v>0</v>
+      </c>
+      <c r="V2" s="3">
+        <v>0</v>
+      </c>
+      <c r="W2" s="3">
+        <v>0</v>
+      </c>
+      <c r="X2" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AK2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AR2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AY2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ2" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA2" s="3"/>
+      <c r="BB2" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>